<commit_message>
Auditoría A9, evidencia consolidada, correcciones y log de ejecución
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRA8AMApDbLs5bWnCDcYVN
</commit_message>
<xml_diff>
--- a/research/05_MODELOS_DE_NEGOCIO.xlsx
+++ b/research/05_MODELOS_DE_NEGOCIO.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="149">
   <si>
     <t xml:space="preserve">05 — Modelos de negocio (A5) · fecha 2026-10-19 · moneda USD</t>
   </si>
@@ -131,7 +131,7 @@
     <t xml:space="preserve">Ticket medio por suscripción</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope RG 1125: UVA 3.000 por emisión (≈USD 4.300, E5011, sujeto del tope a confirmar).</t>
+    <t xml:space="preserve">Tope RG 1125 por inversor: UVA 3.000 por emisión (≈USD 4.300) y UVA 10.000 total (art. 148, E9005).</t>
   </si>
   <si>
     <t xml:space="preserve">recurr</t>
@@ -254,6 +254,15 @@
     <t xml:space="preserve">Sin ancla. Ref. briq.mx cobra dictamen legal MXN 17.000 (A2).</t>
   </si>
   <si>
+    <t xml:space="preserve">coloc_op</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comisión de colocación del operador autorizado (M1, la paga el emisor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin tarifa pública. Ref. colocación FF Total Assets V 0,89% (E5016) y ON Vitalcan ~1% (E8003).</t>
+  </si>
+  <si>
     <t xml:space="preserve">fijo_m1</t>
   </si>
   <si>
@@ -434,7 +443,7 @@
     <t xml:space="preserve">fijo ÷ contribución por campaña</t>
   </si>
   <si>
-    <t xml:space="preserve">fee orig. + prep + estructuración + arancel + 2% colocación del operador (SUPUESTO)</t>
+    <t xml:space="preserve">fee orig. + prep + estructuración + arancel + colocación del operador</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidad M2 (resto de supuestos en escenario BASE). Resultado operativo anual en USD.</t>
@@ -960,7 +969,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -1446,21 +1455,47 @@
         <v>77</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>250000</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>90000</v>
+        <v>28</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.02</v>
       </c>
       <c r="G19" s="4" t="s">
         <v>20</v>
       </c>
       <c r="H19" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1490,7 +1525,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>12</v>
@@ -1502,12 +1537,12 @@
         <v>14</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B2" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$3</f>
@@ -1522,12 +1557,12 @@
         <v>30000000</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">B2/Supuestos!$D$6</f>
@@ -1542,12 +1577,12 @@
         <v>15000</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Supuestos!$D$6</f>
@@ -1562,12 +1597,12 @@
         <v>2000</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Supuestos!$D$4+Supuestos!$D$5</f>
@@ -1582,12 +1617,12 @@
         <v>0.1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">B3*B4*B5</f>
@@ -1602,12 +1637,12 @@
         <v>3000000</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B3/Supuestos!$D$7</f>
@@ -1622,12 +1657,12 @@
         <v>3750</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">B7*Supuestos!$D$8</f>
@@ -1642,12 +1677,12 @@
         <v>187500</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7*Supuestos!$D$9</f>
@@ -1662,12 +1697,12 @@
         <v>3000</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B7*Supuestos!$D$10</f>
@@ -1682,12 +1717,12 @@
         <v>11250</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$11</f>
@@ -1702,12 +1737,12 @@
         <v>45000</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$12</f>
@@ -1722,12 +1757,12 @@
         <v>45000</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">B2*Supuestos!$D$15</f>
@@ -1742,12 +1777,12 @@
         <v>30000</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">Supuestos!$D$16</f>
@@ -1762,12 +1797,12 @@
         <v>200000</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">SUM(B8:B14)</f>
@@ -1782,12 +1817,12 @@
         <v>521750</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B6-B15</f>
@@ -1802,12 +1837,12 @@
         <v>2478250</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">IF(B6=0,0,B16/B6)</f>
@@ -1822,12 +1857,12 @@
         <v>0.826083333333333</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">(Supuestos!$D$8+Supuestos!$D$9+Supuestos!$D$10)/(Supuestos!$D$6*Supuestos!$D$7)+(Supuestos!$D$11+Supuestos!$D$12)/Supuestos!$D$3+Supuestos!$D$15</f>
@@ -1842,12 +1877,12 @@
         <v>0.010725</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B5-B18</f>
@@ -1862,12 +1897,12 @@
         <v>0.089275</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B20" s="8" t="str">
         <f aca="false">IF(B19&lt;=0,"NUNCA (contribución negativa)",Supuestos!$D$16/B19)</f>
@@ -1882,12 +1917,12 @@
         <v>2240268.83225987</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B21" s="13" t="str">
         <f aca="false">IF(ISNUMBER(B20),B20/Supuestos!$D$3,"n/a")</f>
@@ -1902,12 +1937,12 @@
         <v>2.24026883225987</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">Supuestos!$D$4+Supuestos!$D$13/Supuestos!$D$3+Supuestos!$D$14</f>
@@ -1922,7 +1957,7 @@
         <v>0.08815</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1951,7 +1986,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>12</v>
@@ -1963,12 +1998,12 @@
         <v>14</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B2" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$3</f>
@@ -1983,12 +2018,12 @@
         <v>30000000</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">Supuestos!$D$2</f>
@@ -2003,12 +2038,12 @@
         <v>30</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Supuestos!$D$3</f>
@@ -2023,12 +2058,12 @@
         <v>1000000</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Supuestos!$D$17</f>
@@ -2043,12 +2078,12 @@
         <v>0.035</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">B3*B4*B5</f>
@@ -2063,12 +2098,12 @@
         <v>1050000</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$18*1</f>
@@ -2083,12 +2118,12 @@
         <v>180000</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">B6+B7</f>
@@ -2103,12 +2138,12 @@
         <v>1230000</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$11</f>
@@ -2123,12 +2158,12 @@
         <v>45000</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">Supuestos!$D$2*Supuestos!$D$12</f>
@@ -2143,12 +2178,12 @@
         <v>45000</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B2*Supuestos!$D$15/2</f>
@@ -2163,32 +2198,32 @@
         <v>15000</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B12" s="8" t="n">
-        <f aca="false">Supuestos!$D$19</f>
+        <f aca="false">Supuestos!$D$20</f>
         <v>250000</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">Supuestos!$E$19</f>
+        <f aca="false">Supuestos!$E$20</f>
         <v>150000</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">Supuestos!$F$19</f>
+        <f aca="false">Supuestos!$F$20</f>
         <v>90000</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">SUM(B9:B12)</f>
@@ -2203,12 +2238,12 @@
         <v>195000</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">B8-B13</f>
@@ -2223,12 +2258,12 @@
         <v>1035000</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">IF(B8=0,0,B14/B8)</f>
@@ -2243,12 +2278,12 @@
         <v>0.841463414634146</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">Supuestos!$D$3*Supuestos!$D$17+Supuestos!$D$18-Supuestos!$D$11-Supuestos!$D$12-Supuestos!$D$3*Supuestos!$D$15/2</f>
@@ -2263,47 +2298,47 @@
         <v>37500</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B17" s="13" t="str">
-        <f aca="false">IF(B16&lt;=0,"NUNCA",Supuestos!$D$19/B16)</f>
+        <f aca="false">IF(B16&lt;=0,"NUNCA",Supuestos!$D$20/B16)</f>
         <v>NUNCA</v>
       </c>
       <c r="C17" s="13" t="n">
-        <f aca="false">IF(C16&lt;=0,"NUNCA",Supuestos!$E$19/C16)</f>
+        <f aca="false">IF(C16&lt;=0,"NUNCA",Supuestos!$E$20/C16)</f>
         <v>23.0769230769231</v>
       </c>
       <c r="D17" s="13" t="n">
-        <f aca="false">IF(D16&lt;=0,"NUNCA",Supuestos!$F$19/D16)</f>
+        <f aca="false">IF(D16&lt;=0,"NUNCA",Supuestos!$F$20/D16)</f>
         <v>2.4</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B18" s="11" t="n">
-        <f aca="false">(Supuestos!$D$17*Supuestos!$D$3+Supuestos!$D$18+Supuestos!$D$13)/Supuestos!$D$3+Supuestos!$D$14+0.02</f>
+        <f aca="false">(Supuestos!$D$17*Supuestos!$D$3+Supuestos!$D$18+Supuestos!$D$13)/Supuestos!$D$3+Supuestos!$D$14+Supuestos!$D$19</f>
         <v>0.31515</v>
       </c>
       <c r="C18" s="11" t="n">
-        <f aca="false">(Supuestos!$E$17*Supuestos!$E$3+Supuestos!$E$18+Supuestos!$E$13)/Supuestos!$E$3+Supuestos!$E$14+0.02</f>
+        <f aca="false">(Supuestos!$E$17*Supuestos!$E$3+Supuestos!$E$18+Supuestos!$E$13)/Supuestos!$E$3+Supuestos!$E$14+Supuestos!$E$19</f>
         <v>0.10515</v>
       </c>
       <c r="D18" s="11" t="n">
-        <f aca="false">(Supuestos!$F$17*Supuestos!$F$3+Supuestos!$F$18+Supuestos!$F$13)/Supuestos!$F$3+Supuestos!$F$14+0.02</f>
+        <f aca="false">(Supuestos!$F$17*Supuestos!$F$3+Supuestos!$F$18+Supuestos!$F$13)/Supuestos!$F$3+Supuestos!$F$14+Supuestos!$F$19</f>
         <v>0.06915</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2331,17 +2366,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B4" s="14" t="n">
         <v>0.03</v>
@@ -2565,12 +2600,12 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>1</v>
@@ -2740,12 +2775,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>300</v>
@@ -2942,12 +2977,12 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B34" s="15" t="n">
         <v>100000</v>
@@ -2970,23 +3005,23 @@
         <v>2</v>
       </c>
       <c r="B35" s="8" t="n">
-        <f aca="false">$A35*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A35*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-151250</v>
       </c>
       <c r="C35" s="8" t="n">
-        <f aca="false">$A35*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A35*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-144125</v>
       </c>
       <c r="D35" s="8" t="n">
-        <f aca="false">$A35*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A35*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-132250</v>
       </c>
       <c r="E35" s="8" t="n">
-        <f aca="false">$A35*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A35*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-108500</v>
       </c>
       <c r="F35" s="8" t="n">
-        <f aca="false">$A35*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A35*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-61000</v>
       </c>
     </row>
@@ -2995,23 +3030,23 @@
         <v>4</v>
       </c>
       <c r="B36" s="8" t="n">
-        <f aca="false">$A36*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A36*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-152500</v>
       </c>
       <c r="C36" s="8" t="n">
-        <f aca="false">$A36*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A36*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-138250</v>
       </c>
       <c r="D36" s="8" t="n">
-        <f aca="false">$A36*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A36*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-114500</v>
       </c>
       <c r="E36" s="8" t="n">
-        <f aca="false">$A36*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A36*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-67000</v>
       </c>
       <c r="F36" s="8" t="n">
-        <f aca="false">$A36*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A36*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>28000</v>
       </c>
     </row>
@@ -3020,23 +3055,23 @@
         <v>8</v>
       </c>
       <c r="B37" s="8" t="n">
-        <f aca="false">$A37*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A37*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-155000</v>
       </c>
       <c r="C37" s="8" t="n">
-        <f aca="false">$A37*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A37*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-126500</v>
       </c>
       <c r="D37" s="8" t="n">
-        <f aca="false">$A37*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A37*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-79000</v>
       </c>
       <c r="E37" s="8" t="n">
-        <f aca="false">$A37*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A37*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>16000</v>
       </c>
       <c r="F37" s="8" t="n">
-        <f aca="false">$A37*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A37*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>206000</v>
       </c>
     </row>
@@ -3045,23 +3080,23 @@
         <v>12</v>
       </c>
       <c r="B38" s="8" t="n">
-        <f aca="false">$A38*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A38*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-157500</v>
       </c>
       <c r="C38" s="8" t="n">
-        <f aca="false">$A38*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A38*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-114750</v>
       </c>
       <c r="D38" s="8" t="n">
-        <f aca="false">$A38*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A38*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-43500</v>
       </c>
       <c r="E38" s="8" t="n">
-        <f aca="false">$A38*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A38*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>99000</v>
       </c>
       <c r="F38" s="8" t="n">
-        <f aca="false">$A38*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A38*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>384000</v>
       </c>
     </row>
@@ -3070,23 +3105,23 @@
         <v>20</v>
       </c>
       <c r="B39" s="8" t="n">
-        <f aca="false">$A39*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A39*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-162500</v>
       </c>
       <c r="C39" s="8" t="n">
-        <f aca="false">$A39*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A39*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-91250</v>
       </c>
       <c r="D39" s="8" t="n">
-        <f aca="false">$A39*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A39*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>27500</v>
       </c>
       <c r="E39" s="8" t="n">
-        <f aca="false">$A39*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A39*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>265000</v>
       </c>
       <c r="F39" s="8" t="n">
-        <f aca="false">$A39*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A39*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>740000</v>
       </c>
     </row>
@@ -3095,23 +3130,23 @@
         <v>30</v>
       </c>
       <c r="B40" s="8" t="n">
-        <f aca="false">$A40*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A40*(B$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-B$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-168750</v>
       </c>
       <c r="C40" s="8" t="n">
-        <f aca="false">$A40*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A40*(C$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-C$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>-61875</v>
       </c>
       <c r="D40" s="8" t="n">
-        <f aca="false">$A40*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A40*(D$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-D$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>116250</v>
       </c>
       <c r="E40" s="8" t="n">
-        <f aca="false">$A40*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A40*(E$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-E$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>472500</v>
       </c>
       <c r="F40" s="8" t="n">
-        <f aca="false">$A40*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$19</f>
+        <f aca="false">$A40*(F$34*Supuestos!$E$17+Supuestos!$E$18-Supuestos!$E$11-Supuestos!$E$12-F$34*Supuestos!$E$15/2)-Supuestos!$E$20</f>
         <v>1185000</v>
       </c>
     </row>

</xml_diff>